<commit_message>
Sprint 5 Day 32: Capital Allocation Report
</commit_message>
<xml_diff>
--- a/output/cashflow_intelligence.xlsx
+++ b/output/cashflow_intelligence.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H3"/>
+  <dimension ref="A1:I3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -469,6 +469,11 @@
           <t>deleveraging_flag</t>
         </is>
       </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>capital_allocation_label</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -501,6 +506,11 @@
       <c r="H2" t="b">
         <v>1</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -532,6 +542,11 @@
       </c>
       <c r="H3" t="b">
         <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>Reinvestor</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>